<commit_message>
fix: update panel-aviso-corte template and tests
</commit_message>
<xml_diff>
--- a/tests/aviso.xlsx
+++ b/tests/aviso.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HIDROAA\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HIDROAA\Desktop\antares\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DEA146-A5D4-418F-A887-A07CB9216BAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFBF745-E8D5-489D-A954-3F3DD9EC6FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>ID</t>
   </si>
@@ -49,9 +49,6 @@
     <t>CUADRANTE A-12</t>
   </si>
   <si>
-    <t>Mantenimiento Preventivo de Redes</t>
-  </si>
-  <si>
     <t>1002</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>CUADRANTE B-05</t>
   </si>
   <si>
-    <t>Reparación de Tubería Matriz</t>
-  </si>
-  <si>
     <t>1003</t>
   </si>
   <si>
@@ -76,9 +70,6 @@
     <t>CUADRANTE C-08</t>
   </si>
   <si>
-    <t>Mejora de Presión en la Zona</t>
-  </si>
-  <si>
     <t>1004</t>
   </si>
   <si>
@@ -91,9 +82,6 @@
     <t>CUADRANTE D-11</t>
   </si>
   <si>
-    <t>Conexión de Nuevas Redes</t>
-  </si>
-  <si>
     <t>1005</t>
   </si>
   <si>
@@ -125,6 +113,30 @@
   </si>
   <si>
     <t>CUADRANTE D-12</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R104</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R105</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R106</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R107</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R108</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R109</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R110</t>
+  </si>
+  <si>
+    <t>Trabajos de mejoramiento del reservorio R111</t>
   </si>
 </sst>
 </file>
@@ -492,7 +504,7 @@
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="5" max="5" width="43.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -526,63 +538,63 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -591,61 +603,61 @@
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>